<commit_message>
Update bulkhead and aerodynamic analysis spreadsheets
Revised Bulkhead analysis.xlsx and ESTYCTRL HRD-02 Aerodynamic and dynamic design spreadsheet with updated data or calculations.
</commit_message>
<xml_diff>
--- a/Bulkhead analysis.xlsx
+++ b/Bulkhead analysis.xlsx
@@ -1,20 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D11DF1B-1BBE-4439-90F3-DF8F3E7B2031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="28680" yWindow="1770" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="30">
   <si>
     <t>Length</t>
   </si>
@@ -70,9 +84,6 @@
     <t>t</t>
   </si>
   <si>
-    <t>kg/mm^2</t>
-  </si>
-  <si>
     <t>0.1 Mpa</t>
   </si>
   <si>
@@ -86,14 +97,35 @@
   </si>
   <si>
     <t>altura</t>
+  </si>
+  <si>
+    <t>plywood</t>
+  </si>
+  <si>
+    <t>Depends on type of wood</t>
+  </si>
+  <si>
+    <t>Density</t>
+  </si>
+  <si>
+    <t>kg/m3</t>
+  </si>
+  <si>
+    <t>Mass bulkhead</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>gr</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="171" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -142,7 +174,7 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -166,20 +198,26 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>180976</xdr:rowOff>
+      <xdr:rowOff>6351</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>593705</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>123826</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>314305</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>130176</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="International pressure units - WIKA blog"/>
+        <xdr:cNvPr id="2" name="Picture 1" descr="International pressure units - WIKA blog">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
         </xdr:cNvPicPr>
@@ -199,8 +237,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="2695575" y="180976"/>
-          <a:ext cx="3965555" cy="2228850"/>
+          <a:off x="3752850" y="6351"/>
+          <a:ext cx="3965555" cy="2114550"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -221,33 +259,45 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>175375</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>6350</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>111875</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>277215</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>38580</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>607415</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>152880</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="5" name="Group 4"/>
+        <xdr:cNvPr id="5" name="Group 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGrpSpPr/>
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2724150" y="2080375"/>
-          <a:ext cx="3649065" cy="1768205"/>
+          <a:off x="3838575" y="1740650"/>
+          <a:ext cx="3645890" cy="1669780"/>
           <a:chOff x="2695575" y="2080375"/>
           <a:chExt cx="3649065" cy="1768205"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:pic>
         <xdr:nvPicPr>
-          <xdr:cNvPr id="3" name="Picture 2"/>
+          <xdr:cNvPr id="3" name="Picture 2">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
           <xdr:cNvPicPr>
             <a:picLocks noChangeAspect="1"/>
           </xdr:cNvPicPr>
@@ -270,7 +320,13 @@
       </xdr:pic>
       <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
-          <xdr:cNvPr id="4" name="TextBox 3"/>
+          <xdr:cNvPr id="4" name="TextBox 3">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
           <xdr:cNvSpPr txBox="1"/>
         </xdr:nvSpPr>
         <xdr:spPr>
@@ -315,20 +371,26 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>247650</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>514350</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>191088</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>9840</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>457788</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>47940</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5"/>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -341,8 +403,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2686050" y="3848100"/>
-          <a:ext cx="4210638" cy="2257740"/>
+          <a:off x="3648075" y="3695700"/>
+          <a:ext cx="4210638" cy="2140265"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -355,9 +417,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -395,9 +457,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -432,7 +494,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -467,7 +529,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -640,21 +702,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:F51"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.140625" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.1796875" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" customWidth="1"/>
+    <col min="3" max="3" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -666,7 +728,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>0</v>
       </c>
@@ -677,7 +739,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>1</v>
       </c>
@@ -689,169 +751,211 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6">
+        <v>1200</v>
+      </c>
+      <c r="D6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7">
+        <f>C6/C4</f>
+        <v>8.5932927653666766E-2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10">
+        <v>1750</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C11" s="1">
+        <f>C10*(0.1/14.5)</f>
+        <v>12.068965517241381</v>
+      </c>
+      <c r="D11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13">
+        <f>C11/C7</f>
+        <v>140.44634398914718</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B15" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
         <v>3</v>
       </c>
-      <c r="C5">
-        <v>30</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="C16">
+        <v>45.9</v>
+      </c>
+      <c r="D16" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7">
-        <v>1200</v>
-      </c>
-      <c r="D7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8">
-        <f>C7/C4</f>
-        <v>8.5932927653666766E-2</v>
-      </c>
-      <c r="D8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11">
-        <v>1750</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C12" s="1">
-        <f>C11*(0.1/14.5)</f>
-        <v>12.068965517241381</v>
-      </c>
-      <c r="D12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14">
-        <f>C12/C8</f>
-        <v>140.44634398914718</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C17">
-        <v>55</v>
+        <f>2.375*25.4</f>
+        <v>60.324999999999996</v>
       </c>
       <c r="D17" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C18">
-        <f>2.375*25.4</f>
-        <v>60.324999999999996</v>
+        <f>(PI()/4)*((C17^2)-C16^2)</f>
+        <v>1203.462169656945</v>
       </c>
       <c r="D18" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19">
+        <f>(C17-C16)/2</f>
+        <v>7.2124999999999986</v>
+      </c>
+      <c r="D19" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B19" t="s">
-        <v>16</v>
-      </c>
-      <c r="C19">
-        <f>(PI()/4)*((C18^4)-C17^4)</f>
-        <v>3214214.2983454713</v>
-      </c>
-      <c r="D19" t="s">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20">
+        <f>C6/C18</f>
+        <v>0.99712315871305546</v>
+      </c>
+      <c r="D20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B23" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23">
+        <v>750</v>
+      </c>
+      <c r="D23" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25">
         <v>5</v>
       </c>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B20" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20">
-        <f>(C18-C17)/2</f>
-        <v>2.6624999999999979</v>
-      </c>
-      <c r="D20" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21">
-        <f>0.2232/C20</f>
-        <v>8.3830985915493025E-2</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="D25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27">
+        <f>C25/C20</f>
+        <v>5.0144257069039373</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28">
+        <f>(C18/(1000*1000))*(C3/1000)*C23</f>
+        <v>4.5129831362135442E-2</v>
+      </c>
+      <c r="D28" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C29">
+        <f>C28*1000</f>
+        <v>45.129831362135441</v>
+      </c>
+      <c r="D29" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B32" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C22">
-        <f>C21+(0.1/102)</f>
-        <v>8.4811378072355767E-2</v>
-      </c>
-      <c r="D22" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
+      <c r="C32" t="s">
         <v>19</v>
       </c>
-      <c r="C24" t="s">
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="C33" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C25" t="s">
+    <row r="35" spans="2:6" x14ac:dyDescent="0.35">
+      <c r="E35" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="E35" t="s">
-        <v>22</v>
       </c>
       <c r="F35" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B36">
         <v>22.751999999999999</v>
       </c>
@@ -866,7 +970,7 @@
         <v>196.85</v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B37">
         <v>23.564</v>
       </c>
@@ -881,7 +985,7 @@
         <v>146.04999999999998</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B39">
         <f>24.134+0.02</f>
         <v>24.154</v>
@@ -891,7 +995,7 @@
         <v>613.51159999999993</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B40" s="1">
         <f>C40/25.4</f>
         <v>24.178346456692914</v>
@@ -900,12 +1004,12 @@
         <v>614.13</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B42" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B43">
         <v>14.207000000000001</v>
       </c>
@@ -914,12 +1018,12 @@
         <v>360.8578</v>
       </c>
     </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:6" x14ac:dyDescent="0.35">
       <c r="C44">
         <v>360.66</v>
       </c>
     </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B46">
         <v>0.97</v>
       </c>
@@ -928,7 +1032,7 @@
         <v>3.8188976377952759E-2</v>
       </c>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B47">
         <v>0.16</v>
       </c>
@@ -937,7 +1041,7 @@
         <v>6.2992125984251976E-3</v>
       </c>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B48">
         <v>0.31</v>
       </c>
@@ -946,7 +1050,7 @@
         <v>1.2204724409448819E-2</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B49">
         <v>0.31</v>
       </c>
@@ -955,7 +1059,7 @@
         <v>1.2204724409448819E-2</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B50">
         <v>0.17</v>
       </c>
@@ -964,7 +1068,7 @@
         <v>6.6929133858267724E-3</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B51">
         <v>0.73</v>
       </c>

</xml_diff>

<commit_message>
Update analysis and design Excel files
Revised 'Bulkhead analysis.xlsx' and 'ESTYCTRL HRD-02 Diseño Aerodinámico y dinámico Rev.1 (1).xlsx' with new data or calculations. Review changes for updated analysis results.
</commit_message>
<xml_diff>
--- a/Bulkhead analysis.xlsx
+++ b/Bulkhead analysis.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D11DF1B-1BBE-4439-90F3-DF8F3E7B2031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BBA5F02-5341-46D5-B292-6554B1077972}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1770" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="31">
   <si>
     <t>Length</t>
   </si>
@@ -118,6 +118,9 @@
   </si>
   <si>
     <t>gr</t>
+  </si>
+  <si>
+    <t>ya</t>
   </si>
 </sst>
 </file>
@@ -283,8 +286,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="3838575" y="1740650"/>
-          <a:ext cx="3645890" cy="1669780"/>
+          <a:off x="4559300" y="1769225"/>
+          <a:ext cx="3649065" cy="1698355"/>
           <a:chOff x="2695575" y="2080375"/>
           <a:chExt cx="3649065" cy="1768205"/>
         </a:xfrm>
@@ -707,7 +710,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.1796875" customWidth="1"/>
-    <col min="2" max="2" width="12.7265625" customWidth="1"/>
+    <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -824,7 +827,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>15</v>
       </c>
@@ -836,7 +839,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>16</v>
       </c>
@@ -848,7 +851,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>17</v>
       </c>
@@ -860,7 +863,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>8</v>
       </c>
@@ -871,13 +874,16 @@
       <c r="D20" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="E20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
         <v>25</v>
       </c>
@@ -888,12 +894,12 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>8</v>
       </c>
@@ -904,7 +910,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>12</v>
       </c>
@@ -913,7 +919,7 @@
         <v>5.0144257069039373</v>
       </c>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>27</v>
       </c>
@@ -925,7 +931,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
       <c r="C29">
         <f>C28*1000</f>
         <v>45.129831362135441</v>
@@ -934,7 +940,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B32" t="s">
         <v>18</v>
       </c>

</xml_diff>